<commit_message>
align submission tables with original problem requirements
</commit_message>
<xml_diff>
--- a/results/表1_温度.xlsx
+++ b/results/表1_温度.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -640,7 +640,7 @@
     <row r="1" ht="14.1" customHeight="1" s="4">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>时间\到药材中心的距离</t>
+          <t>时间/s\到药材中心的距离/cm</t>
         </is>
       </c>
       <c r="B1" s="2" t="n">
@@ -664,19 +664,19 @@
         <v>100</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>28</v>
+        <v>28.0001</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>28</v>
+        <v>28.0003</v>
       </c>
       <c r="D2" s="5" t="n">
         <v>28.004</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>28.033</v>
+        <v>28.0327</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>28.177</v>
+        <v>28.1801</v>
       </c>
     </row>
     <row r="3" ht="14.1" customHeight="1" s="4">
@@ -684,19 +684,19 @@
         <v>300</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>28.041</v>
+        <v>28.0408</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>28.063</v>
+        <v>28.0635</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>28.151</v>
+        <v>28.1514</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>28.368</v>
+        <v>28.3681</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>28.84</v>
+        <v>28.8489</v>
       </c>
     </row>
     <row r="4" ht="14.1" customHeight="1" s="4">
@@ -704,10 +704,10 @@
         <v>600</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>28.453</v>
+        <v>28.4533</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>28.536</v>
+        <v>28.5361</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>28.804</v>
@@ -716,7 +716,7 @@
         <v>29.316</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>30.152</v>
+        <v>30.1653</v>
       </c>
     </row>
     <row r="5" ht="14.1" customHeight="1" s="4">
@@ -724,19 +724,19 @@
         <v>900</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>29.324</v>
+        <v>29.3243</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>29.458</v>
+        <v>29.4583</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>29.875</v>
+        <v>29.8755</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>30.616</v>
+        <v>30.6162</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>31.714</v>
+        <v>31.7305</v>
       </c>
     </row>
     <row r="6">
@@ -744,19 +744,19 @@
         <v>1200</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>30.543</v>
+        <v>30.5427</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>30.71</v>
+        <v>30.7098</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>31.222</v>
+        <v>31.2224</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>32.113</v>
+        <v>32.1126</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>33.408</v>
+        <v>33.4277</v>
       </c>
     </row>
     <row r="7">
@@ -764,19 +764,19 @@
         <v>1500</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>31.996</v>
+        <v>31.9957</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>32.187</v>
+        <v>32.1868</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>32.766</v>
+        <v>32.7661</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>33.746</v>
+        <v>33.7463</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>35.101</v>
+        <v>35.1204</v>
       </c>
     </row>
     <row r="8">
@@ -784,19 +784,19 @@
         <v>1800</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>33.575</v>
+        <v>33.5754</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>33.772</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>34.364</v>
+        <v>34.3642</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>35.362</v>
+        <v>35.3622</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>36.765</v>
+        <v>36.7856</v>
       </c>
     </row>
   </sheetData>

</xml_diff>